<commit_message>
feat: Fix Lorry generation mapping and COA remain lifetime auto-check
</commit_message>
<xml_diff>
--- a/n系統報表產生/N系料小包-地點代號對照表.xlsx
+++ b/n系統報表產生/N系料小包-地點代號對照表.xlsx
@@ -14,12 +14,12 @@
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="27">
   <si>
     <t>短地點</t>
   </si>
@@ -111,6 +111,13 @@
   </si>
   <si>
     <t>F22P2B</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>15P7</t>
+  </si>
+  <si>
+    <t>L1400251</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -470,7 +477,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="13.75" customWidth="1"/>
@@ -658,6 +665,17 @@
         <v>1</v>
       </c>
     </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16">
+        <v>1570</v>
+      </c>
+      <c r="C16" t="s">
+        <v>26</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>